<commit_message>
Resample Excel excluding team/seed papers; update generator script
New sample of 10 papers drawn from 744 non-team papers (pool excludes
the 27 TROPESS seed papers whose paper_id == a team_paper_id).
Mix: 7 Data Usage, 2 Review Paper, 1 Simple Citation.
</commit_message>
<xml_diff>
--- a/TROPESS_sample_10_papers.xlsx
+++ b/TROPESS_sample_10_papers.xlsx
@@ -628,63 +628,63 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ammonia emissions and depositions over the contiguous United States derived from IASI and CrIS using the directional derivative approach</t>
+          <t>State of Wildfires 2024–2025</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Zitong Li; Kang Sun; Kaiyu Guan; Sheng Wang; Bin Peng; L. Clarisse; M. Van Damme; P. Coheur; K. Cady-Pereira; M. Shephard; M. Zondlo; Daniel Moore</t>
+          <t>Douglas I. Kelley; Chantelle A. Burton; F. Di Giuseppe; Matthew W. Jones; M. L. Barbosa; Esther Brambleby; J. McNorton; Zhongwei Liu; A. Bradley; Katie Blackford; E. Burke; A. Ciavarella; Enza Di Tomaso; Jonathan M. Eden; I. J. M. Ferreira; L. Fiedler; Andrew J. Hartley; Theodore R Keeping; Seppe Lampe; A. Lombardi; G. Mataveli; Yuquan Qu; P. S. Silva; Fiona R. Spuler; Carmen B. Steinmann; M. A. Torres-Vázquez; Renata Veiga; D. van Wees; Jakob B. Wessel; Emily Wright; B. Bilbao; Mathieu L. Bourbonnais; Cong Gao; C. D. Di Bella; K. Dintwe; Victoria M. Donovan; Sarah Harris; E. Kukavskaya; A. B. N’Dri; C. Santín; G. Selaya; Johan Sjöström; J. Abatzoglou; N. Andela; Rachel Carmenta; E. Chuvieco; Louis Giglio; D. Hamilton; S. Hantson; Sarah Meier; M. Parrington; M. Sadegh; J. San-Miguel-Ayanz; Fernando Sedano; Marco Turco; G. R. van der Werf; S. Veraverbeke; L. Anderson; Hamish Clarke; P. Fernandes; Crystal A. Kolden</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Atmospheric Chemistry and Physics</t>
+          <t>Earth System Science Data</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>10.5194/acp-26-703-2026</t>
+          <t>10.5194/essd-17-5377-2025</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/acp-26-703-2026</t>
+          <t>https://doi.org/10.5194/essd-17-5377-2025</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1f7484592d508fea344bc32760fc8cf2b62b68bf</t>
+          <t>83e94004ccf4de8d78313e86066006426be42bb0</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Data Usage</t>
+          <t>Review Paper</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>The provided engagement_level is 'Data Usage'. The abstract explicitly states the paper 'estimated NH3 fluxes ... using satellite observations from the ... Cross-track Infrared Sounder (CrIS),' which is a TROPESS instrument, confirming active data usage.</t>
+          <t>The abstract describes the paper as an 'annual report' that 'systematically tracks global and regional fire activity,' indicating a review or survey nature.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>algorithm</t>
+          <t>science</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>The abstract states the paper 'estimated NH3 fluxes ... using satellite observations from ... CrIS ... by applying a directional derivative approach,' indicating a focus on retrieval methodology and data processing from satellite instruments.</t>
+          <t>The paper systematically tracks and analyzes global wildfire activity, causes, and future projections, contributing to the understanding of Earth science phenomena related to climate and wildfires.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Trace Gas Products</t>
+          <t>Wildfire &amp; Biomass Burning Emissions</t>
         </is>
       </c>
       <c r="N2" s="2" t="n"/>
@@ -711,12 +711,13 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>Abstract. Atmospheric ammonia (NH3), primarily emitted from agriculture, poses significant threats to ecosystems, climate, and human health through nitrogen deposition and secondary aerosol formation. NH3 flux estimates remain highly uncertain due to limited direct observations and complex emission–deposition processes. Here, we estimated NH3 fluxes over the contiguous United States using satellite observations from the Infrared Atmospheric Sounding Interferometer (IASI, 2008–2022) and Cross-track Infrared Sounder (CrIS, 2012–2022) by applying a directional derivative approach. Our results highlight major agricultural emission hotspots, including the San Joaquin Valley in California, the Snake River Valley in Idaho, the Texas panhandle, the Great Plains, Southeastern Pennsylvania, and Eastern North Carolina. NH3 removal is predominantly driven by deposition near source areas rather than chemical transformation, with strong sinks in vegetation-dense regions such as forests, grasslands, shrublands, and wetlands. Seasonal flux variations show peaks in warm months and lower values in winter, driven by temperature-dependent volatilization from livestock production and fertilizer application. Compared with bottom-up inventory, satellite-based estimates capture general spatial and seasonal patterns, while also revealing additional insights into key flux hotspots and peak periods. CrIS consistently reports higher fluxes than IASI, especially in spring, reflecting differences in their overpass times. Combining IASI (morning overpass) and CrIS (midday overpass) observations enables a better understanding of diurnal NH3 flux dynamics. These findings provide critical insights into NH3 spatiotemporal variabilities, complementing inventory-based approaches and informing nitrogen management and environmental policy, particularly in regions with limited ground-based monitoring.</t>
+          <t xml:space="preserve">Abstract. Climate change is increasing the frequency and intensity of extreme wildfires globally, yet our understanding of these high-impact events remains uneven and shaped by media attention and regional research biases. The State of Wildfires project systematically tracks global and regional fire activity of each annual fire season, analyses the causes of prominent extreme wildfire events, and projects the likelihood of similar events occurring in future climate scenarios. This, its second annual report, covers the March 2024 to February 2025 fire season. During the 2024–2025 fire season, fire-related carbon (C) emissions totalled 2.2 Pg C, 9 % above average and the sixth highest on record since 2003, despite below-average global burned area (BA). Extreme fire seasons in South America's rainforests, dry forests, and wetlands and in Canada's boreal forests pushed up the global C emissions total. Fire C emissions were over 4 times above average in Bolivia, 3 times above average in Canada, and ∼ 50 % above average in Brazil and Venezuela. Wildfires in 2024–2025 caused 100 fatalities in Nepal, 34 in South Africa, and 31 in Los Angeles, with additional fatalities reported in Canada, Côte d'Ivoire, Portugal, and Türkiye. The Eaton and Palisades fires in Southern California caused 150 000 evacuations and USD 140 billion in damages. Communities in Brazil, Bolivia, Southern California, and northern India were exposed to fine particulate matter at concentrations 13–60 times WHO's daily air quality standards. We evaluated the causes and predictability of four extreme wildfire episodes from the 2024–2025 fire season, including in Northeast Amazonia (January–March 2024), the Pantanal–Chiquitano border regions of Brazil and Bolivia (August–September 2024), Southern California (January 2025), and the Congo Basin (July–August 2024). Anomalous weather created conditions for these regional extremes, while fuel availability and human ignitions shaped spatial patterns and temporal fire dynamics. In the three tropical regions, prolonged drought was the dominant fire enabler, whereas in California, extreme heat, wind, and antecedent fuel build-up were compounding enablers. Our attribution analyses show that climate change made extreme fire weather in Northeast Amazonia 30–70 times more likely, increasing BA roughly 4-fold compared to a scenario without climate change. In the Pantanal–Chiquitano, fire weather was 4–5 times more likely, with 35-fold increases in BA. Meanwhile, our analyses suggest that BA was 25 times higher in Southern California due to climate change. The Congo Basin's fire weather was 3–8 times more likely with climate change, with a 2.7-fold increase in BA. Socioeconomic changes since the pre-industrial period, including land-use change, also likely increased BA in Northeast Amazonia. Our models project that events on the scale of 2024–2025 will become up to 57 %, 34 %, and 50 % more frequent than in the modern era in Northeast Amazonia, the Pantanal–Chiquitano, and the Congo Basin, respectively, under a medium–high scenario (SSP370) by 2100. Climate action can limit the added risk, with frequency increases held to below 15 % in all three regions under a strong mitigation scenario (SSP126). In Southern California, the future trajectory of extreme fire likelihood remains highly uncertain due to poorly constrained climate–vegetation–fire interactions influencing fuel moisture, though our models suggest that risk may decline in future. This annual report from the State of Wildfires project integrates and advances cutting-edge fire observations and modelling with regional expertise to track changing global wildfire hazard, guiding policy and practice towards improved preparedness, mitigation, adaptation, and societal benefit. Thirteen new datasets and model codebases presented in this work are available from the State of Wildfires Project's Zenodo community, including updated annual statistics on wildfire extent (Jones et al., 2025; https://doi.org/10.5281/zenodo.15525674), outputs from modelling of fire causality using PoF model (Di Giuseppe, 2025; https://doi.org/10.24433/CO.8570224.v1) and codebase for the extreme event attribution/projections model, ConFLAME (Barbosa et al., 2025a, https://doi.org/10.5281/zenodo.16790787).
+</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>0.95</v>
+        <v>0.975</v>
       </c>
       <c r="W2" s="2" t="n">
         <v>0.85</v>
@@ -729,12 +730,12 @@
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Atmosphere to Surface Profiles of Water‐Vapor Isotopes and Meteorological Conditions Over the Northeast Greenland Ice Sheet</t>
+          <t>Comprehensive 24-hour ground-level ozone monitoring: Leveraging machine learning for full-coverage estimation in East Asia.</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Kevin S. Rozmiarek; L. J. Dietrich; Bruce H. Vaughn; Michael S. Town; B. Markle; Valerie Morris; H. Steen‐Larsen; X. Fettweis; Chloe Brashear; H. Bennett; Tyler R. Jones</t>
+          <t>Yejin Kim; Seohui Park; Hyunyoung Choi; Jungho Im</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -742,26 +743,26 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Journal of Geophysical Research: Atmospheres</t>
+          <t>Journal of Hazardous Materials</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>10.1029/2024JD042719</t>
+          <t>10.1016/j.jhazmat.2025.137369</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1029/2024JD042719</t>
+          <t>https://doi.org/10.1016/j.jhazmat.2025.137369</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>1ec6918a68304479c16da6fb375a4a507824e453</t>
+          <t>548aed1e75f393415b16a091cab24bf8ce569154</t>
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
@@ -770,42 +771,34 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>The paper presents novel aircraft measurements of water vapor isotopes and cites two TROPESS team papers, including one on 'Characterization and evaluation of AIRS-based estimates of tropospheric water vapor isotopes,' strongly suggesting the use of AIRS data for comparison or contextualization of their new dataset.</t>
+          <t>The paper develops an ozone estimation model using 'Himawari-8 brightness temperature,' which is a satellite-derived data source, to address limitations in satellite-derived ozone concentration estimation.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>This paper presents a novel dataset of water vapor isotopes to understand how 'water vapor interacts with surface snow' and imprints an 'isotopic climate signal into the ice sheet,' focusing on Earth science phenomena.</t>
+          <t>The paper focuses on developing a 'novel all-sky O3 estimation model based on a light gradient boosting machine' to obtain gap-free ozone estimates, which is a development in retrieval methodology.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Validation &amp; Intercomparison</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
+          <t>Trace Gas Products</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n"/>
+      <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Characterization and evaluation of AIRS-based estimates of the deuterium content of water vapor</t>
+          <t>Balance of Emission and Dynamical Controls on Ozone During the Korea-United States Air Quality Campaign From Multiconstituent Satellite Data Assimilation</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>tropess_team_d530907b9585e4df</t>
+          <t>tropess_team_8ce74f979a112381</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -820,12 +813,12 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>On polar ice sheets, water vapor interacts with surface snow, and through the exchange of water molecules, imprints an isotopic climate signal into the ice sheet. This exchange is not well understood due to sparse observations in the atmosphere. There are currently no published vertical profiles of water isotopes above ice sheets that span the planetary boundary layer and portions of the free troposphere. Here, we present a novel data set of water‐vapor isotopes ( δ18 ${\delta }^{18}$ O, δ $\delta $ D, dxs $dxs$ ) and meteorological variables taken by fixed‐wing uncrewed aircraft on the northeast Greenland Ice Sheet (GIS). During June–July (2022), we collected 104 profiles of water‐vapor isotopes and meteorological variables up to 1,500 m above ground level. Concurrently, surface snow samples were collected at 12‐hr intervals, allowing connection to surface‐snow processes. We pair observations with modeling output from a regional climate model as well as an atmospheric transport and water‐isotope distillation model. Climate model output of mean temperature and specific humidity agrees well with observations, with a mean difference of +0.095°C and −0.043 g/kg (−2.91%), respectively. We find evidence that along an air parcel pathway, the distillation model is not removing enough water prior to onsite arrival. Below the mean temperature inversion ( ∼ ${\sim} $ 200 m), water‐isotope observations indicate a kinetic fractionating process, likely the result of mixing sublimated vapor from the ice sheet surface along with an unknown fraction of katabatic wind vapor. Modeled dxs $dxs$ does not agree well with observations, a result that requires substantial future analysis of kinetic fractionation processes along the entire moisture pathway.</t>
+          <t>Cloud cover often hinders satellite-derived ozone (O3) concentration estimation, leading to incomplete spatial coverage. To address this limitation and obtain gap-free hourly ground-level O3 estimates, this study developed a novel all-sky O3 estimation model based on a light gradient boosting machine, combining clear- (cLearGBM) and cloudy-sky (cLoudGBM) models. Unlike earlier studies focusing mainly on daytime, this study provides comprehensive O3 variations over a full 24-h cycle at an hourly 2 km resolution. The all-sky O3 estimation model was developed using Himawari-8 brightness temperature (BT) as a key input, alongside other satellite-derived variables, meteorological variables, and auxiliary parameters, with ground-based O3 observations serving as the dependent variable. The models were evaluated using three 10-fold cross-validation methods (random, spatial, and temporal), showing high estimation accuracy (cLearGBM: coefficient of determination (R2) = 0.90, root mean square error (RMSE) = 8.77 ppb; cLoudGBM: R2 = 0.87, RMSE = 9.44 ppb). Notably, BT data improved the accuracy and spatial resolution of the O3 estimates. The estimated ground-level O3 distribution followed a typical diurnal pattern across the study area, with urban regions showing higher O3 concentrations during the day and rural areas exhibiting higher concentrations at night. Compared to the Copernicus Atmosphere Monitoring Service reanalysis data, the proposed model offered a representation of East Asia that was 40 times better spatial resolution and 2.26 times more accurate when evaluated against in-situ observations. The 24-h ground-level O3 data for East Asia provided by this study is expected to serve as a valuable foundation for applied research and to support effective O3 pollution management.</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr"/>
       <c r="V3" s="3" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="W3" s="3" t="n">
         <v>0.85</v>
@@ -838,39 +831,39 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Validation of MUSES NH3 observations from AIRS and CrIS against aircraft measurements from DISCOVER-AQ and a surface network in the Magic Valley</t>
+          <t>Origins and characterization of CO and O3 in the African upper troposphere</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>K. Cady-Pereira; X. Guo; R. Wang; A. Leytem; C. Calkins; E. Berry; K. Sun; M. Muller; A. Wisthaler; V. Payne; M. Shephard; M. Zondlo; V. Kantchev</t>
+          <t>V. Lannuque; B. Sauvage; B. Barret; H. Clark; G. Athier; D. Boulanger; J. Cammas; J. Cousin; A. Fontaine; E. Le Flochmoën; P. Nédélec; H. Petetin; Isabelle Pfaffenzeller; S. Rohs; H. Smit; Pawel Wolff; V. Thouret</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Atmos. Meas. Tech.</t>
+          <t>Atmospheric Chemistry and Physics</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>10.5194/amt-17-15-2024</t>
+          <t>10.5194/ACP-21-14535-2021</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/amt-17-15-2024</t>
+          <t>https://acp.copernicus.org/articles/21/14535/2021/acp-21-14535-2021.pdf</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>tropess_team_a5e48c6037f49001</t>
+          <t>b9e541129c70983267974f00762e94a037197899</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -879,36 +872,36 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>The paper directly validates MUSES NH3 observations derived from AIRS and CrIS against aircraft and surface measurements.</t>
+          <t>The paper actively uses 'measurements from the IASI instrument onboard the Metop-A satellite' to characterize CO and O3, and IASI is an infrared sounder measuring trace gases, making it TROPESS-adjacent.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>algorithm</t>
+          <t>science</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>The primary focus is on the 'Validation of MUSES NH3 observations from AIRS and CrIS against aircraft measurements', which falls under satellite product validation.</t>
+          <t>This paper characterizes the distributions and seasonality of CO and O3 in the African upper troposphere and explores their sources and origins, which is an investigation of atmospheric processes.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Validation &amp; Intercomparison</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="n"/>
+          <t>Trace Gas Products</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>High-resolution tropospheric carbon monoxide profiles retrieved from CrIS and TROPOMI</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>tropess_team_1d89a3ab71c53f9c</t>
+        </is>
+      </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
           <t>True</t>
@@ -921,15 +914,16 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>Abstract. Ammonia is a significant precursor of PM2.5 particles and thus contributes to poor air quality in many regions. Furthermore, ammonia concentrations are rising due to the increase of large-scale, intensive agricultural activities, which are often accompanied by greater use of fertilizers and concentrated animal feedlots. Ammonia is highly reactive and thus highly variable and difficult to measure. Satellite-based instruments, such as the Atmospheric Infrared Sounder (AIRS) and the Cross-Track Infrared Sounder (CrIS), have been shown to provide much greater temporal and spatial coverage of ammonia distribution and variability than is possible with in situ networks or aircraft campaigns, but the validation of these data is limited. Here we evaluate MUSES (multi-spectra, multi-species, multi-sensors) ammonia retrievals from AIRS and CrIS against ammonia measurements from aircraft in the California Central Valley and in the Colorado Front Range. These are small datasets taken over high-source regions under very different conditions: winter in California and summer in Colorado. Direct comparisons of the surface values of the retrieved profiles are biased very low in California (∼ 40 ppbv) and slightly high in Colorado (∼ 4 ppbv). This bias appears to be primarily due to smoothing error, since applying the instrument operator effectively reduces the bias to zero; even after the smoothing error is accounted for, the average uncertainty at the surface is in the 20 %–30 % range. We also compare 3 years of CrIS ammonia against an in situ network in the Magic Valley in Idaho We show that CrIS ammonia captures both the seasonal signal and the spatial variability in the Magic Valley, although it is biased low here also. In summary, this analysis substantially adds to the validation record but also points to the need for more validation under many different conditions and at higher altitudes.</t>
+          <t xml:space="preserve">Abstract. Between December 2005 and 2013, the In-service Aircraft for a Global Observing System (IAGOS) program produced almost daily in situ measurements of CO and O3 between Europe and southern Africa. IAGOS data combined with measurements from the IASI instrument onboard the Metop-A satellite (2008–2013) are used to characterize meridional distributions and seasonality of CO and O3 in the African upper troposphere (UT). The FLEXPART particle dispersion model and the SOFT-IO model which combines the FLEXPART model with CO emission inventories are used to explore the sources and origins of the observed transects of CO and O3. We focus our analysis on two main seasons: December to March (DJFM) and June to October (JJASO). These seasons have been defined according to the position of Intertropical Convergence Zone (ITCZ), determined using in situ measurements from IAGOS. During both seasons, the UT CO meridional transects are characterized by maximum mixing ratios located 10° from the position of the ITCZ above the dry regions inside the hemisphere of the strongest Hadley cell (132 to 165 ppb at 0–5° N in DJFM and 128 to 149 ppb at 3–7° S in JJASO), and decreasing values south- and north-ward. The O3 meridional transects are characterized by mixing ratio minima of ~ 42–54 ppb at the ITCZ (10–16° S in DJFM and 5–8° N in JJASO) framed by local maxima (~ 53–71 ppb) coincident with the wind shear zones North and South of the ITCZ. O3 gradients are strongest in the hemisphere of the strongest Hadley cell. IASI UT O3 distributions in DJFM have revealed that the maxima are a part of a crescent-shaped O3 plume above the Atlantic Ocean around the Gulf of Guinea. CO emitted at the surface is transported towards the ITCZ by the trade winds and then convectively uplifted. Once in the upper troposphere, CO enriched air masses are transported away from the ITCZ by the upper branches of the Hadley cells and accumulate within the zonal wind shear zones where the maximum CO mixing ratios are found. Anthropogenic and fires both contribute, by the same order of magnitude, to the CO budget of the African upper troposphere. Local fires have the highest contribution, drive the location of the observed UT CO maxima, and are related to the following transport pathway: CO emitted at the surface is transported towards the ITCZ by the trade winds and further convectively uplifted. Then UT CO enriched air masses are transported away from the ITCZ by the upper branches of the Hadley cells and accumulate within the zonal wind shear zones where the maxima are located. Anthropogenic CO contribution is mostly from Africa during the entire year, with a low seasonal variability, and is related to similar transport circulation than fire air masses. There is also a large contribution from Asia in JJASO related to the fast convective uplift of polluted air masses in the Asian monsoon region which are further westward transported by the tropical easterly jet (TEJ) and the Asian monsoon anticyclone (AMA). O3 minima correspond to air masses that were recently uplifted from the surface where mixing ratios are low at the ITCZ. The O3 maxima correspond to old high altitude air masses uplifted from either local or long distance area of high O3 precursor emissions (Africa and South America during all the year, South Asia mainly in JJASO), and must be created during transport by photochemistry. This analysis of meridional transects contribute to a better understanding of distributions of CO and O3 in the intertropical African upper troposphere and the processes which drive these distributions. Therefore, it provides a solid basis for comparison and improvement of models and satellite products in order to get the good O3 for the good reasons.
+</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>0.425</v>
+        <v>0.95</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="X4" s="2" t="inlineStr"/>
       <c r="Y4" s="2" t="inlineStr"/>
@@ -939,39 +933,39 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Global atmospheric inversion of the anthropogenic NH3 emissions over 2019–2022 using the LMDZ-INCA chemistry transport model and the IASI NH3 observations</t>
+          <t>Assessing the Responses of Aviation-Related SO2 and NO2 Emissions to COVID-19 Lockdown Regulations in South Africa</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Pramod Kumar; G. Broquet; D. Hauglustaine; M. Beaudor; L. Clarisse; M. Van Damme; P. Coheur; A. Cozic; Bo-Yan Zheng; Beatriz Revilla Romero; Antony Delavois; P. Ciais</t>
+          <t>L. Shikwambana; Mahlatse Kganyago</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Atmospheric Chemistry and Physics</t>
+          <t>Remote Sensing</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>10.5194/acp-25-12379-2025</t>
+          <t>10.3390/rs13204156</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/acp-25-12379-2025</t>
+          <t>https://doi.org/10.3390/rs13204156</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>21cc611cd506b39ba49f4af6f21acfb42021eeb5</t>
+          <t>fa8c09f6b5014602308903b9539a36a5f35b3142</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -980,7 +974,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>The paper actively uses data from a closely related infrared sounder, stating, "We use IASI-ANNI-NH3-v4 satellite observations" for global atmospheric inversion.</t>
+          <t>The paper assesses responses of aviation-related SO2 and NO2 emissions, a common application for satellite data. It cites 'Air Quality Response in China Linked to the 2019 Novel Coron', a TROPESS team paper likely using satellite data for air quality analysis during COVID-19.</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -990,24 +984,24 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>The paper uses satellite observations and a chemistry transport model to provide 'atmospheric inversion estimates of the global NH3 emissions,' focusing on understanding an Earth science phenomenon.</t>
+          <t>The paper assesses the responses of aviation-related SO2 and NO2 emissions to COVID-19 lockdown regulations, focusing on changes in anthropogenic emissions and their environmental impact.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Trace Gas Products</t>
+          <t>Air Quality &amp; Megacity Studies</t>
         </is>
       </c>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Validation of MUSES NH3 observations from AIRS and CrIS against aircraft measurements from DISCOVER-AQ and a surface network in the Magic Valley</t>
+          <t>Air Quality Response in China Linked to the 2019 Novel Coronavirus (COVID-19) Lockdown</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>tropess_team_a5e48c6037f49001</t>
+          <t>tropess_team_1bc49f64ec00d99e</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
@@ -1022,13 +1016,12 @@
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract. Ammonia (NH3) emissions have been on a continuous rise due to extensive fertilizer usage in agriculture and increasing production of manure and livestock. However, the current global-to-national NH3 emission inventories exhibit large uncertainties. We provide atmospheric inversion estimates of the global NH3 emissions over 2019–2022 at 1.27° × 2.5° horizontal and daily (at 10 d scale) resolution. We use IASI-ANNI-NH3-v4 satellite observations, simulations of NH3 concentrations with the chemistry transport model LMDZ-INCA, and the finite difference mass-balance approach for inversions of global NH3 emissions. We take advantage of the averaging kernels provided in the IASI-ANNI-NH3-v4 dataset by applying them consistently to the LMDZ-INCA NH3 simulations for comparison to the observations and then to invert emissions. The average global anthropogenic NH3 emissions over 2019–2022 are estimated as ∼97 (94–100) Tg yr−1, which is ∼61 % (∼55 %–65 %) higher than the prior Community Emissions Data System (CEDS) inventory's anthropogenic NH3 emissions and significantly higher than two other global inventories: CAMS's anthropogenic NH3 emissions (by a factor of ∼1.8) and the Calculation of AMmonia Emissions in ORCHIDEE (CAMEO) agricultural and natural soil NH3 emissions (by ∼1.4 times). The global and regional budgets are mostly within the range of other inversion estimates. The analysis provides confidence in their seasonal variability and continental- to regional-scale budgets. Our analysis shows a rise in NH3 emissions by ∼5 % to ∼37 % during the COVID-19 lockdowns in 2020 over different regions compared to the same-period emissions in 2019. However, this rise is probably due to a decrease in atmospheric NH3 sinks due to the decline in NOx and SO2 emissions during the lockdowns.
-</t>
+          <t>Aircraft emit harmful substances, such as carbon dioxide (CO2), water vapour (H2O), nitrogen oxides (NOx), sulphur oxides (SOx), particulates, and other trace compounds. These emissions degrade air quality and can deteriorate human health and negatively impact climate change. Airports are the nucleus of the ground and low-altitude emissions from aircraft during approach, landing, take-off, and taxi. During the global lockdown due to the COVID-19 pandemic, tight restrictions of the movement were imposed, leading to temporary closures of airports globally. In this study, we look at the variability of emissions at two major airports in South Africa, namely the OR Tambo international airport (FAOR) and the Cape Town international airport (FACT). Trend analysis of aircraft movements, i.e., departures and arrivals, showed a sharp decline at the two airports coinciding with the lockdowns to prevent the spread of the COVID-19. Consequently, a decrease in NO2 emissions by 70.45% (12.6 × 10−5 mol/m2) and 64.58% (11.6 × 10−5 mol/m2) at FAOR and FACT were observed, respectively. A noticeable SO2 emission decline was also observed, particularly over FAOR during the lockdown period in South Africa. Overall, this study observed that the global lockdown regulations had a positive impact on the air quality, causing a brief decline in emissions from commercial aviation at the South African major airports.</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr"/>
       <c r="V5" s="3" t="n">
-        <v>0.925</v>
+        <v>0.95</v>
       </c>
       <c r="W5" s="3" t="n">
         <v>0.85</v>
@@ -1041,12 +1034,12 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Elucidating the Effects of COVID-19 Lockdowns in the UK on the O3-NOx-VOC Relationship</t>
+          <t>Short‐Lived Air Pollutants and Climate Forcers Through the Lens of the COVID‐19 Pandemic</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Rayne Holland; Katya Seifert; Eric Saboya; M. Khan; R. Derwent; D. Shallcross</t>
+          <t>Yuan Wang; Chenchong Zhang; E. Pennington; Liyin He; Jiani Yang; Xueying Yu; Yangfan Liu; J. Seinfeld</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -1054,35 +1047,35 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Atmosphere</t>
+          <t>Reviews of Geophysics</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>10.3390/atmos15050607</t>
+          <t>10.1029/2022RG000773</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.mdpi.com/2073-4433/15/5/607/pdf?version=1715858127</t>
+          <t>https://doi.org/10.1029/2022RG000773</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>bb9a7c7155493741831c1e535a55c58eaf2b20d3</t>
+          <t>8a237b82d923d9a874eb27ef0042a1c7177ba712</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Data Usage</t>
+          <t>Review Paper</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>The paper investigates the response of ozone and its precursors to emission changes during COVID-19 lockdowns, a topic frequently addressed with satellite data. It cites the TROPESS team paper 'Air Quality Response in China Linked to the 2019 Novel Coron,' which uses satellite observations for air quality analysis, suggesting a connection to TROPESS data or methodologies.</t>
+          <t>The paper is explicitly described as a 'Review Paper' and its abstract indicates a synthesis of progress in understanding atmospheric changes.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1092,7 +1085,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>The paper investigates the response of ozone concentrations to changes in its precursors to understand the O3-NOx-VOC relationship.</t>
+          <t>The paper synthesizes progress in understanding changes in short-lived atmospheric constituents and their climate impacts in response to emission reductions.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1102,12 +1095,12 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1132,12 +1125,12 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>The unprecedented reductions in anthropogenic emissions over the COVID-19 lockdowns were utilised to investigate the response of ozone (O3) concentrations to changes in its precursors across various UK sites. Ozone, volatile organic compounds (VOCs) and NOx (NO+NO2) data were obtained for a 3-year period encompassing the pandemic period (January 2019–December 2021), as well as a pre-pandemic year (2017), to better understand the contribution of precursor emissions to O3 fluctuations. Compared with pre-lockdown levels, NO and NO2 declined by up to 63% and 42%, respectively, over the lockdown periods, with the most significant changes in pollutant concentrations recorded across the urban traffic sites. O3 levels correspondingly increased by up to 30%, consistent with decreases in the [NO]/[NO2] ratio for O3 concentration response. Analysis of the response of O3 concentrations to the NOx reductions suggested that urban traffic, suburban background and suburban industrial sites operate under VOC-limited regimes, while urban background, urban industrial and rural background sites are NOx-limited. This was in agreement with the [VOC]/[NOx] ratios determined for the London Marylebone Road (LMR; urban traffic) site and the Chilbolton Observatory (CO; rural background) site, which produced values below and above 8, respectively. Conversely, [VOC]/[NOx] ratios for the London Eltham (LE; suburban background) site indicated NOx-sensitivity, which may suggest the [VOC]/[NOx] ratio for O3 concentration response may have had a slight NOx-sensitive bias. Furthermore, O3 concentration response with [NO]/[NO2] and [VOC]/[NOx] were also investigated to determine their relevance and accuracy in identifying O3-NOx-VOC relationships across UK sites. While the results obtained via utilisation of these metrics would suggest a shift in photochemical regime, it is likely that variation in O3 during this period was primarily driven by shifts in oxidant (OX; NO2 + O3) equilibrium as a result of decreasing NO2, with increased O3 transported from Europe likely having some influence.</t>
+          <t>Dramatic reductions in anthropogenic emissions during the lockdowns of the COVID‐19 pandemic provide an unparalleled opportunity to assess responses of the Earth system to human activities. Here, we synthesize the latest progress in understanding changes in short‐lived atmospheric constituents, that is, aerosols, ozone (O3), nitrogen oxides (NOx), and methane (CH4), in response to COVID‐19 induced emission reductions and the associated climate impacts on regional and global scales. The large‐scale emission reduction in the transportation sector reduced near‐surface particulate and ozone concentrations, with certain regional enhancements modulated by atmospheric oxidizing capacity and abnormal meteorological conditions. The methane increase during the pandemic is a combined effect of fluctuations in methane emissions and chemical sinks. Global net radiative forcing of all short‐lived species was found to be small, but regionally, aerosol radiative impacts during the lockdowns were discernible near China and India. Aerosol microphysical effects on clouds and precipitation were reported from modeling assessments only, except for observed reductions in aircraft contrails. There exist moderate climatic impacts of the pandemic on regional surface temperature, atmospheric circulations, and ecosystems, mainly over populous and polluted areas. Novel methodologies emerge in the pandemic‐related research to achieve the synergy between observations from multiple platforms and model simulations and to overcome the enormous hurdles and sophistication in detection and attribution studies. The insight gained from COVID‐19 research concerning the complex interplay between emission, chemistry, and meteorology, as well as the unexpected climate forcing‐responses relationships, underscores future challenges for cleaning up the air and alleviating the adverse impacts of global warming.</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>0.825</v>
+        <v>1</v>
       </c>
       <c r="W6" s="2" t="n">
         <v>0.85</v>
@@ -1150,12 +1143,12 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Global reanalysis products cannot reproduce seasonal and diurnal cycles of tropospheric ozone in the Congo Basin</t>
+          <t>Comparing Sentinel-5P TROPOMI NO2 column observations with the CAMS regional air quality ensemble</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>I. Vieira; H. Verbeeck; F. Meunier; M. Peaucelle; Thomas Sibret; Lodewijk Lefevre; A. Cheesman; Flossie Brown; S. Sitch; José Mbifo; P. Boeckx; M. Bauters</t>
+          <t>J. Douros; H. Eskes; J. van Geffen; K. F. Boersma; S. Compernolle; G. Pinardi; A. Blechschmidt; V. Peuch; A. Colette; P. Veefkind</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -1163,26 +1156,26 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Atmospheric Environment</t>
+          <t>Geoscientific Model Development</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>10.1016/j.atmosenv.2023.119773</t>
+          <t>10.5194/gmd-16-509-2023</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://biblio.ugent.be/publication/01GZ3H4VCNVGG26YEF1Y7MHXW9/file/01H18Y1PBCKE8P7BGJHB4E8QJB.pdf</t>
+          <t>https://gmd.copernicus.org/articles/16/509/2023/gmd-16-509-2023.pdf</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>3c44713654c1ffbb1a47607184e9c84240a46ac8</t>
+          <t>0146348e325b125bdb171790a8bc422f351925c4</t>
         </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
@@ -1191,22 +1184,22 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>The title explicitly states the paper evaluates 'Global reanalysis products' for tropospheric ozone, and it cites 'Updated tropospheric chemistry reanalysis and emission estim,' confirming active engagement with a TROPESS-related reanalysis product.</t>
+          <t>The title explicitly states 'Comparing Sentinel-5P TROPOMI NO2 column observations' and the abstract indicates these datasets are used 'to test high-resolution regional-scale air quality (AQ) models,' which constitutes active data usage of a TROPESS-adjacent instrument.</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>This study investigates the seasonal and diurnal cycles of tropospheric ozone in the Congo Basin and assesses the performance of global reanalysis products in representing these cycles, focusing on atmospheric processes.</t>
+          <t>The paper focuses on comparing Sentinel-5P TROPOMI NO2 observations with a regional air quality model ensemble, which involves validating model performance against satellite data.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Atmospheric Chemistry &amp; Reanalysis</t>
+          <t>Tropospheric Composition Retrievals</t>
         </is>
       </c>
       <c r="N7" s="3" t="n"/>
@@ -1233,15 +1226,16 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Tropospheric ozone (O 3 ) is a secondary pollutant and a greenhouse gas with a positive radiative forcing . Many studies have documented its negative impacts on plant growth and human health. Historically, studies have focused on determining levels of exposure in mid- and high-latitude regions. In the tropics, high O 3 concentrations are expected due to large concurrent and future precursor emissions. In Africa, seasonal biomass burning (from both natural and anthropogenic fires) during the dry season plays a crucial role in O 3 precursor production. However, O 3 observational studies in tropical Africa are currently missing. To fill this major knowledge gap, we established in November 2019 a continuous monitoring of near-surface O 3 in the Congo Basin at the Yangambi research centre in the Democratic Republic of the Congo. Using this unique dataset in the heart of the second-largest tropical forest in the world, we assessed the ability of current remote sensing products to capture the magnitude and temporal dynamics of in situ tropospheric O 3 concentrations, especially O 3 concentration variation between dry and wet seasons until March of 2022. We compared near-surface atmospheric O 3 measurements collected in Yangambi and four different reanalysis products: European Centre for Medium-Range Weather Forecasts Reanalysis (ECMWF) v5 (ERA5), Copernicus Atmospheric Monitoring Service reanalysis (CAMSRA), Modern-Era Retrospective Analysis for Research and Applications version 2 (MERRA-2) and Japanese Reanalysis (JRA-55). The results show that reanalysis products overestimated the magnitude of near-surface O 3 across the region with a mean bias of 27.3 ppbv, 19.9 ppbv, 10.8 ppbv and 1.0 ppbv for ERA5, CAMSRA, MERRA-2 and JRA-55, respectively. ERA5 and CAMSRA reanalysis were the only products able to capture, to some extent, the observed annual variation, showing higher O 3 concentrations during dry season months, despite the inability to reproduce the daily cycle of near-surface O 3 . • The first-ever dataset of near-surface ozone was collected in the core of the African tropical forests. • It fills a critical gap in a relevant area as ozone has been thought to reach large concentrations in central Africa. • Access the ability of state-of-the-art reanalysis products to capture the magnitude and temporal dynamics of in situ O3. • The reanalysis products fail to reproduce the seasonality and the daily cycles of tropospheric ozone.</t>
+          <t xml:space="preserve">Abstract. The Sentinel-5P TROPOspheric Monitoring Instrument (TROPOMI) instrument, launched in October 2017, provides unique observations of atmospheric trace gases at a high resolution of about 5 km, with near-daily global coverage, resolving individual sources like thermal powerplants, industrial complexes, fires, medium-scale towns, roads, and shipping routes. Even though Sentinel-5P (S5P) is a global mission, these datasets are especially well suited to test high-resolution regional-scale air quality (AQ) models and provide valuable input for emission inversion systems. In Europe, the Copernicus Atmosphere Monitoring Service (CAMS) has implemented an operational regional AQ forecasting capability based on an ensemble of several European models, available at a resolution of 0.1∘ × 0.1∘. In this paper, we present comparisons between TROPOMI observations of nitrogen dioxide (NO2) and the CAMS AQ forecasts and analyses of NO2. We discuss the different ways of making these comparisons and present quantitative results in the form of maps for individual days, summer and winter months, and a time series for European subregions and cities between May 2018 and March 2021. The CAMS regional products generally capture the fine-scale daily and averaged features observed by TROPOMI in much detail. In summer, the comparison shows a close agreement between TROPOMI and the CAMS ensemble NO2 tropospheric columns with a relative difference of up to 15 % for most European cities. In winter, however, we find a significant discrepancy in the column amounts over much of Europe, with relative differences up to 50 %. The possible causes for these differences are discussed, focusing on the possible impact of retrieval and modeling errors. Apart from comparisons with the CAMS ensemble, we also present results for comparisons with the individual CAMS models for selected months. Furthermore, we demonstrate the importance of the free tropospheric contribution to the estimation of the tropospheric column and thus include profile information from the CAMS configuration of the ECMWF's (European Centre for Medium-Range Weather Forecasts) global integrated model above 3 km altitude in the comparisons. We also show that replacing the global 1∘ × 1∘ a priori information in the retrieval by the regional 0.1∘ × 0.1∘ resolution profiles of CAMS leads to significant changes in the TROPOMI-retrieved tropospheric column, with typical increases at the emission hotspots up to 30 % and smaller increases or decreases elsewhere. As a spinoff, we present a new TROPOMI NO2 level 2 (L2) data product for Europe, based on the replacement of the original TM5-MP generated global a priori profile by the regional CAMS ensemble profile. This European NO2 product is compared with ground-based remote sensing measurements of six Pandora instruments of the Pandonia Global Network and nine Multi-AXis Differential Optical Absorption Spectroscopy (MAX-DOAS) instruments. As compared to the standard S5P tropospheric NO2 column data, the overall bias of the new product for all except two stations is 5 % to 12 % smaller, owing to a reduction in the multiplicative bias. Compared to the CAMS tropospheric NO2 columns, dispersion and correlation parameters with respect to the standard data are, however, superior.
+</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr"/>
       <c r="V7" s="3" t="n">
-        <v>0.425</v>
+        <v>0.975</v>
       </c>
       <c r="W7" s="3" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="X7" s="3" t="inlineStr"/>
       <c r="Y7" s="3" t="inlineStr"/>
@@ -1251,75 +1245,71 @@
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Air pollution modulates trends and variability of the global methane budget</t>
+          <t>Updating Chinese SO2 emissions with surface observations for regional air-quality modeling over East Asia</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Yuanhong Zhao; Bo-Yan Zheng; M. Saunois; P. Ciais; M. Hegglin; Shengmin Lu; Yifan Li; Philippe Bousquet</t>
+          <t>C. Bae; Hyun Cheol Kim; Byeong-Uk Kim; Younha Kim; J. Woo; Soontae Kim</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Nature</t>
-        </is>
-      </c>
+        <v>2020</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-09004-z</t>
+          <t>10.1016/j.atmosenv.2020.117416</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41586-025-09004-z</t>
+          <t>https://doi.org/10.1016/j.atmosenv.2020.117416</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>fb1ac36ec0907504a22686d1a0eb6fb679eb5757</t>
+          <t>bda48b75b92fe2cf320fd69b3837b7e6434f6ab3</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Data Usage</t>
+          <t>Simple Citation</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>The engagement_level is explicitly stated as "Data Usage", implying active use of TROPESS or closely related satellite retrievals.</t>
+          <t>The abstract describes a top-down emission update system using surface observations to update Chinese SO2 emissions. There is no mention of TROPESS or related satellite data being used.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>The title suggests an investigation into how air pollution affects the global methane budget, focusing on Earth science phenomena.</t>
+          <t>The paper describes the development of 'a top-down emission update system' and 'a data-processing system' for constructing adjustment factors, indicating a focus on methodology development.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Trace Gas Products</t>
+          <t>Air Quality &amp; Megacity Studies</t>
         </is>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Updated tropospheric chemistry reanalysis and emission estimates, TCR-2, for 2005-2018</t>
+          <t>Balance of Emission and Dynamical Controls on Ozone During the Korea-United States Air Quality Campaign From Multiconstituent Satellite Data Assimilation</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>tropess_team_53c33eee24123f48</t>
+          <t>tropess_team_8ce74f979a112381</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1332,13 +1322,17 @@
           <t>TROPESS</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Abstract Anthropogenic emissions in East Asia have changed dramatically in recent years. To measure these changing emissions in support of air-quality modeling, we developed a top-down emission update system using surface observations and a geographical information system spatial-allocation technique. We deploy a data-processing system to construct adjustment factors to prefecture-level SO2 emissions by comparing surface and modeled observations. A case study is conducted over East Asia for 2016 in which we update Chinese SO2 emissions using measurements from around 1500 surface monitoring sites. Model simulations using updated SO2 emissions are improved relative to the existing simulation system (e.g., R = 0.23 to R = 0.8), suggesting that the newly designed system provides an efficient, practical forecast solution. Finally, estimated SO2 emissions are compared with existing emission inventories, agreeing well with recent reports of reduced SO2 emissions from Chinese anthropogenic sources.</t>
+        </is>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr"/>
@@ -1348,39 +1342,35 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Impact of improved representation of volatile organic compound emissions and production of NOx reservoirs on modeled urban ozone production</t>
+          <t>First data set of H2O/HDO columns from the Tropospheric Monitoring Instrument (TROPOMI)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>K. Travis; B. Nault; James H. Crawford; Kelvin H. Bates; Donald R. Blake; R. Cohen; Alan Fried; Samuel R. Hall; L. G. Huey; Young Ro Lee; S. Meinardi; kyung-eun Min; I. Simpson; K. Ullman</t>
+          <t>A. Schneider; T. Borsdorff; J. aan de Brugh; F. Aemisegger; D. Feist; R. Kivi; F. Hase; M. Schneider; J. Landgraf</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Atmospheric Chemistry and Physics</t>
-        </is>
-      </c>
+        <v>2020</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>10.5194/acp-24-9555-2024</t>
+          <t>10.5194/AMT-13-85-2020</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5194/acp-24-9555-2024</t>
+          <t>https://amt.copernicus.org/articles/13/85/2020/amt-13-85-2020.pdf</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>57ea03a44508592faa6087d446ce34b63229ea99</t>
+          <t>d40ba9c0b2a3e96386726583c0f901daaaded0ee</t>
         </is>
       </c>
       <c r="H9" s="3" t="n">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
@@ -1389,17 +1379,17 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>The abstract discusses 'air quality models' and their performance regarding ozone, formaldehyde, and PAN during the KORUS-AQ field study. The citation of a TROPESS team paper on 'Balance of Emission and Dynamical Controls on Ozone' indicates the use of TROPESS-related data or models informed by it for analysis.</t>
+          <t>The paper 'presents a new data set of vertical column densities of H2O and HDO retrieved from... TROPOMI,' indicating active use and development of a product from a TROPESS-adjacent instrument.</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>science</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>The paper investigates the impact of VOC emissions and NOx reservoirs on modeled urban ozone production, which is a study of atmospheric chemistry and air quality.</t>
+          <t>The paper presents a 'new data set of vertical column densities of H2O and HDO retrieved from TROPOMI,' focusing on the methodology of data product generation.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1411,12 +1401,12 @@
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>Balance of Emission and Dynamical Controls on Ozone During the Korea-United States Air Quality Campaign From Multiconstituent Satellite Data Assimilation</t>
+          <t>Characterization and evaluation of AIRS-based estimates of the deuterium content of water vapor</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>tropess_team_8ce74f979a112381</t>
+          <t>tropess_team_d530907b9585e4df</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1431,13 +1421,13 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract. The fraction of urban volatile organic compound (VOC) emissions attributable to fossil fuel combustion has been declining in many parts of the world, resulting in a need to better constrain other anthropogenic sources of these emissions. During the National Institute of Environmental Research (NIER) and National Aeronautics and Space Administration (NASA) Korea-United States Air Quality (KORUS-AQ) field study in Seoul, South Korea, during May–June 2016, air quality models underestimated ozone, formaldehyde, and peroxyacetyl nitrate (PAN), indicating an underestimate of VOCs in the emissions inventory. Here, we use aircraft observations interpreted with the GEOS-Chem chemical transport model (version 13.4.0) to assess the need for increases in VOC emissions and for a revised chemical mechanism to improve treatment of VOC speciation and chemistry. We find that the largest needed VOC emissions increases are attributable to compounds associated with volatile chemical products, liquefied petroleum gas (LPG) and natural gas emissions, and long-range transport. Revising model chemistry to better match observed VOC speciation together with increasing model emissions of underestimated VOC species increased calculated OH reactivity by +2 s−1 and ozone production by +2 ppb h−1. Ozone increased by +6 ppb below 2 km and +9 ppb at the surface, and formaldehyde and acetaldehyde increased by +30 % and +120 % aloft, respectively, all in better agreement with observations. The larger increase in acetaldehyde was attributed to ethanol emissions, which we found to be as important for ozone production as isoprene or alkenes. The increased acetaldehyde significantly reduced the model PAN bias. The need for additional unmeasured VOCs, however, was indicated by a remaining model bias of −0.8 ppb in formaldehyde and a −57 % and −52 % underestimate in higher peroxynitrates (PNs) and alkyl nitrates (ANs), respectively. We added additional chemistry to the model to represent an additional six PNs from observed VOCs but were unable to account for the majority of missing PNs. However, four of these PNs were modeled at concentrations similar to other commonly measured PNs (&gt; 2 % of PAN) indicating that these should be measured in future campaigns and considered from other VOC emission sources (e.g., fires). We hypothesize that emissions of oxygenated VOCs (OVOCs) such as ≥ C5 aldehydes from cooking and/or alkenes associated with volatile chemical products could produce both PNs and ANs and improve remaining model biases. Emerging research on the emissions and chemistry of these species will soon allow for modeling of their impact on local and regional photochemistry.
-</t>
+          <t>Abstract. Global measurements of atmospheric water vapour isotopologues aid to better understand the hydrological cycle and improve global circulation models.
+This paper presents a new data set of vertical column densities of H2O and HDO retrieved from short-wave infrared (2.3  µ m) reflectance measurements by the Tropospheric Monitoring Instrument (TROPOMI) onboard the Sentinel-5 Precursor satellite. TROPOMI features daily global coverage with a spatial resolution of up to 7 km×7 km . The retrieval utilises a profile-scaling approach. The forward model neglects scattering, and strict cloud filtering is therefore necessary. For validation, recent ground-based water vapour isotopologue measurements by the Total Carbon Column Observing Network (TCCON) are employed. A comparison of TCCON δD with ground-based measurements by the Multi-platform remote Sensing of Isotopologues for investigating the Cycle of Atmospheric water (MUSICA) project for data prior to 2014 (where MUSICA data are available) shows a bias in TCCON δD estimates. As TCCON HDO is currently not validated, an overall correction of recent TCCON HDO data is derived based on this finding. The agreement between the corrected TCCON measurements and co-located TROPOMI observations is good with an average bias of ( - 0.2 ± 3 ) × 10 21  molec cm −2 ( (1.1±7.2)  %) in H2O and ( - 2 ± 7 ) × 10 17  molec cm −2 ( ( - 1.1 ± 7.3 )  %) in HDO, which corresponds to a mean bias of ( - 14 ± 17 )  ‰ in a posteriori δD . The bias is lower at low- and mid-latitude stations and higher at high-latitude stations. The use of the data set is demonstrated with a case study of a blocking anticyclone in northwestern Europe in July 2018 using single-overpass data.</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr"/>
       <c r="V9" s="3" t="n">
-        <v>0.875</v>
+        <v>0.85</v>
       </c>
       <c r="W9" s="3" t="n">
         <v>0.85</v>
@@ -1450,39 +1440,35 @@
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Observations of surface CO2 at an urban station in Wuhan, Central China: temporal variations, sources, and sinks</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Wei Liu; Huang Zheng; Feng Ding; Junying Zhang; Yongchun Zhao; Zhuo Xiong; Qian Wu; Linjun Li</t>
-        </is>
-      </c>
+          <t>Forest recovery time following large-scale fires is increasing</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="n">
         <v>2025</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Atmospheric pollution research</t>
+          <t>Nature Ecology &amp; Evolution</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>10.1016/j.apr.2025.102614</t>
+          <t>10.1038/s41559-025-02685-9</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.apr.2025.102614</t>
+          <t>https://doi.org/10.1038/s41559-025-02685-9</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>682c5a213af325b0d3f91653bc9cccf0255ad94a</t>
+          <t>f225180c1f502937a42658c80262d832b6676ad5</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1491,7 +1477,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>The title 'Observations of surface CO2... temporal variations, sources, and sinks' directly relates to atmospheric composition, and the citation of 'Carbon emissions from the 2023 Canadian wildfires' suggests active use or comparison with relevant data.</t>
+          <t>The paper's title indicates an analysis of forest recovery after large-scale fires. Citing 'Carbon emissions from the 2023 Canadian wildfires' suggests the use or direct reference of data related to wildfire impacts or emissions.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1501,12 +1487,12 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>The title indicates the paper focuses on observations and analysis of surface CO2 temporal variations, sources, and sinks in an urban area, which aims to understand atmospheric processes and air quality.</t>
+          <t>The title indicates a study on forest recovery time following large-scale fires, which falls under understanding Earth science phenomena related to ecology and climate.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Air Quality &amp; Megacity Studies</t>
+          <t>Ecology</t>
         </is>
       </c>
       <c r="N10" s="2" t="n"/>
@@ -1534,7 +1520,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>0.425</v>
+        <v>0.35</v>
       </c>
       <c r="W10" s="2" t="n">
         <v>0.5</v>
@@ -1547,39 +1533,39 @@
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Total Column Ozone Retrieval From the Infrared Measurements of a Geostationary Imager</t>
+          <t>Analysis of Long-Term Aerosol Optical Properties Combining AERONET Sunphotometer and Satellite-Based Observations in Hong Kong</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Su Jeong Lee; M. Ahn; S. Ha</t>
+          <t>Xinyu Yu; J. Nichol; Kwonho Lee; Jing Li; M. Wong</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>IEEE Transactions on Geoscience and Remote Sensing</t>
+          <t>Remote Sensing</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>10.1109/TGRS.2019.2901173</t>
+          <t>10.3390/rs14205220</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/TGRS.2019.2901173</t>
+          <t>https://www.mdpi.com/2072-4292/14/20/5220/pdf?version=1666686750</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>7591f65f4e2592330b039b8ca0f95709734b3059</t>
+          <t>1bc5ccc2a5d1edd60d496c23621861c76c6878f3</t>
         </is>
       </c>
       <c r="H11" s="3" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
@@ -1588,42 +1574,42 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>The paper develops a new algorithm for retrieving total column ozone from satellite infrared measurements and cites a TROPESS team paper on tropospheric ozone profile retrievals, indicating engagement with satellite retrieval methodologies.</t>
+          <t>The paper's title and abstract explicitly state it uses 'satellite-based observations' to analyze aerosol optical properties. This, combined with citing a TROPESS team paper on 'Air pollution trends measured from Terra: CO and AOD', confirms active data usage.</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>algorithm</t>
+          <t>science</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>The paper focuses on the development of 'A new algorithm... to retrieve total column ozone (TOZ) from the infrared measurements of a geostationary satellite imager.'</t>
+          <t>The study analyzes seasonal characteristics and long-term variations in aerosol optical parameters in Hong Kong, focusing on understanding atmospheric processes and air quality.</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Trace Gas Products</t>
+          <t>Radiative Transfer &amp; Forward Modeling</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Retrievals of tropospheric ozone profiles from the synergism of AIRS and OMI: methodology and validation</t>
+          <t>Air pollution trends measured from Terra: CO and AOD over industrial, fire-prone, and background regions</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>tropess_team_22b12dfa4c7bc25e</t>
+          <t>tropess_team_88b3da8055d86bb5</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1638,12 +1624,12 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>A new algorithm has been developed to retrieve total column ozone (TOZ) from the infrared measurements of a geostationary satellite imager such as the Advanced Himawari Imager (AHI) aboard Himawari-8 and the advanced meteorological imager flying with the second generation geostationary satellite of South Korea. Based on a nonlinear optimal estimation method, this operational algorithm iteratively retrieves TOZ from AHI thermal measurements under clear-sky conditions as well as over low clouds at 10-min intervals with 6-km spatial resolutions. The first guess for ozone is prepared by combining a monthly climatology with the daily updated TOZ from polar orbiting satellites, while the first guess for the temperature and humidity profiles are from a numerical weather prediction model. AHI contains only one ozone absorption channel ( $9.6~\mu \text{m}$ ), providing information contents (degrees of freedom for signal) of about 0.98 for the ozone retrieval. However, the study shows that the retrieved TOZ successfully captures the temporal and latitudinal variations of ozone flow particularly at mid- and high-latitudes. A validation using the Ozone Monitoring Instrument, Infrared Atmospheric Sounding Interferometer (IASI), and ozonesondes shows that the AHI TOZ are in a good agreement with the three references with mean difference of 2.5%, −0.5%, and 2.6%, respectively. This impressive performance is attributed to the improvements in both first-guess information and the accuracy of the retrieved temperature and humidity profiles. In particular, the good agreement shown in the comparison with the night-time IASI TOZ suggests potential benefits of using the retrieved TOZ for a continuous monitoring of global ozone evolution with high spatial resolution.</t>
+          <t>This study analyzes seasonal characteristics and long-term variations in aerosol optical parameters in Hong Kong from 2006 to 2021 using AERONET data and satellite-based observations based on the extreme-point symmetric mode decomposition (ESMD) model. The dominant aerosol types in Hong Kong are mixed aerosols and urban/industrial aerosols with fine-mode sizes, and slightly absorbing or non-absorbing properties. Aerosol optical depth (AOD), Angstrom exponent (AE) and single scattering albedo (SSA) varied seasonally with a lower AOD but higher AE and SSA in summer, and elevated AOD but lower AE and SSA in spring and winter. The long-term variations show the year 2012 to be a turning point, with an upward trend in AOD and AE before 2012 and then downwards after 2012. However, for SSA, a rising trend was exhibited in both pre- and post-2012 periods, but with a larger gradient in the first period. The ESMD analysis shows shorter-term, non-linear fluctuations in aerosol optical parameters, with alternating increasing and declining trends. The examination of the relationships between AOD and meteorological factors based on the extreme gradient boosting (XGBoost) method shows that the effects of weather conditions on AOD are complex and non-monotonic. A lower relative humidity, higher wind speed in southwest directions and lower temperature are beneficial to the abatement of aerosol loads in Hong Kong. In conclusion, the findings of this study enhance the understanding of aerosol properties and the interactions between aerosol loading and meteorological factors.</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr"/>
       <c r="V11" s="3" t="n">
-        <v>1</v>
+        <v>0.925</v>
       </c>
       <c r="W11" s="3" t="n">
         <v>0.85</v>

</xml_diff>

<commit_message>
Enrich country/all_countries for 487 TROPESS papers via OpenAlex
Re-ran enrich_geographic.py after clearing stale null cache entries.
OpenAlex fallback used for 460 papers. Coverage: 284 → 707/771 papers
now have primary country. Updated sample Excel with populated country
columns.
</commit_message>
<xml_diff>
--- a/TROPESS_sample_10_papers.xlsx
+++ b/TROPESS_sample_10_papers.xlsx
@@ -687,8 +687,16 @@
           <t>Wildfire &amp; Biomass Burning Emissions</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom; Brazil; Germany; Belgium; Netherlands; United States; Switzerland; Spain; France; Canada; China; Argentina; Australia; Russia; Sweden; Portugal</t>
+        </is>
+      </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Carbon emissions from the 2023 Canadian wildfires</t>
@@ -789,8 +797,16 @@
           <t>Trace Gas Products</t>
         </is>
       </c>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>South Korea; United States</t>
+        </is>
+      </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Balance of Emission and Dynamical Controls on Ozone During the Korea-United States Air Quality Campaign From Multiconstituent Satellite Data Assimilation</t>
@@ -890,8 +906,16 @@
           <t>Trace Gas Products</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>France; Belgium; Spain; Germany</t>
+        </is>
+      </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
           <t>High-resolution tropospheric carbon monoxide profiles retrieved from CrIS and TROPOMI</t>
@@ -992,8 +1016,16 @@
           <t>Air Quality &amp; Megacity Studies</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Air Quality Response in China Linked to the 2019 Novel Coronavirus (COVID-19) Lockdown</t>
@@ -1202,8 +1234,16 @@
           <t>Tropospheric Composition Retrievals</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands; Belgium; Germany; United Kingdom; France</t>
+        </is>
+      </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Updated tropospheric chemistry reanalysis and emission estimates, TCR-2, for 2005-2018</t>
@@ -1300,8 +1340,16 @@
           <t>Air Quality &amp; Megacity Studies</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>South Korea; United States</t>
+        </is>
+      </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Balance of Emission and Dynamical Controls on Ozone During the Korea-United States Air Quality Campaign From Multiconstituent Satellite Data Assimilation</t>
@@ -1397,8 +1445,16 @@
           <t>Trace Gas Products</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands; Switzerland; Germany; Finland</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Characterization and evaluation of AIRS-based estimates of the deuterium content of water vapor</t>

</xml_diff>